<commit_message>
Refactor data processing functions and enhance Excel file handling
</commit_message>
<xml_diff>
--- a/output/first10s_events.xlsx
+++ b/output/first10s_events.xlsx
@@ -29282,7 +29282,7 @@
     <row r="996">
       <c r="A996" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B996" t="inlineStr">
@@ -29296,22 +29296,22 @@
         </is>
       </c>
       <c r="D996" t="n">
-        <v>9.300000000000001</v>
+        <v>5.267</v>
       </c>
       <c r="E996" t="n">
-        <v>9.566000000000001</v>
+        <v>5.534</v>
       </c>
       <c r="F996" t="n">
-        <v>0.266</v>
+        <v>0.267</v>
       </c>
       <c r="G996" t="n">
-        <v>0.266</v>
+        <v>0.267</v>
       </c>
     </row>
     <row r="997">
       <c r="A997" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B997" t="inlineStr">
@@ -29321,26 +29321,26 @@
       </c>
       <c r="C997" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D997" t="n">
-        <v>12.7</v>
+        <v>9.534000000000001</v>
       </c>
       <c r="E997" t="n">
-        <v>12.866</v>
+        <v>10.067</v>
       </c>
       <c r="F997" t="n">
-        <v>0.166</v>
+        <v>0.533</v>
       </c>
       <c r="G997" t="n">
-        <v>0.4320000000000001</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="998">
       <c r="A998" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B998" t="inlineStr">
@@ -29350,26 +29350,26 @@
       </c>
       <c r="C998" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D998" t="n">
-        <v>28.033</v>
+        <v>21.634</v>
       </c>
       <c r="E998" t="n">
-        <v>28.366</v>
+        <v>22.034</v>
       </c>
       <c r="F998" t="n">
-        <v>0.333</v>
+        <v>0.4</v>
       </c>
       <c r="G998" t="n">
-        <v>0.7650000000000001</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="999">
       <c r="A999" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B999" t="inlineStr">
@@ -29379,26 +29379,26 @@
       </c>
       <c r="C999" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D999" t="n">
-        <v>32.266</v>
+        <v>42.1</v>
       </c>
       <c r="E999" t="n">
-        <v>33.366</v>
+        <v>42.534</v>
       </c>
       <c r="F999" t="n">
-        <v>1.1</v>
+        <v>0.434</v>
       </c>
       <c r="G999" t="n">
-        <v>1.865</v>
+        <v>1.634</v>
       </c>
     </row>
     <row r="1000">
       <c r="A1000" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1000" t="inlineStr">
@@ -29408,26 +29408,26 @@
       </c>
       <c r="C1000" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1000" t="n">
-        <v>37.733</v>
+        <v>56.234</v>
       </c>
       <c r="E1000" t="n">
-        <v>37.966</v>
+        <v>56.434</v>
       </c>
       <c r="F1000" t="n">
-        <v>0.233</v>
+        <v>0.2</v>
       </c>
       <c r="G1000" t="n">
-        <v>2.098</v>
+        <v>1.834</v>
       </c>
     </row>
     <row r="1001">
       <c r="A1001" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1001" t="inlineStr">
@@ -29441,22 +29441,22 @@
         </is>
       </c>
       <c r="D1001" t="n">
-        <v>50.166</v>
+        <v>61.5</v>
       </c>
       <c r="E1001" t="n">
-        <v>50.966</v>
+        <v>62.534</v>
       </c>
       <c r="F1001" t="n">
-        <v>0.8</v>
+        <v>1.034</v>
       </c>
       <c r="G1001" t="n">
-        <v>2.898000000000001</v>
+        <v>2.868</v>
       </c>
     </row>
     <row r="1002">
       <c r="A1002" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1002" t="inlineStr">
@@ -29466,26 +29466,26 @@
       </c>
       <c r="C1002" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1002" t="n">
-        <v>57.333</v>
+        <v>90.73399999999999</v>
       </c>
       <c r="E1002" t="n">
-        <v>58.266</v>
+        <v>90.934</v>
       </c>
       <c r="F1002" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="G1002" t="n">
-        <v>3.831</v>
+        <v>3.068000000000001</v>
       </c>
     </row>
     <row r="1003">
       <c r="A1003" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1003" t="inlineStr">
@@ -29499,22 +29499,22 @@
         </is>
       </c>
       <c r="D1003" t="n">
-        <v>62.433</v>
+        <v>122.767</v>
       </c>
       <c r="E1003" t="n">
-        <v>63.366</v>
+        <v>123.1</v>
       </c>
       <c r="F1003" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.333</v>
       </c>
       <c r="G1003" t="n">
-        <v>4.764</v>
+        <v>3.401000000000001</v>
       </c>
     </row>
     <row r="1004">
       <c r="A1004" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1004" t="inlineStr">
@@ -29528,22 +29528,22 @@
         </is>
       </c>
       <c r="D1004" t="n">
-        <v>82</v>
+        <v>125.934</v>
       </c>
       <c r="E1004" t="n">
-        <v>82.40000000000001</v>
+        <v>126.1</v>
       </c>
       <c r="F1004" t="n">
-        <v>0.4</v>
+        <v>0.166</v>
       </c>
       <c r="G1004" t="n">
-        <v>5.164000000000001</v>
+        <v>3.567000000000001</v>
       </c>
     </row>
     <row r="1005">
       <c r="A1005" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1005" t="inlineStr">
@@ -29553,26 +29553,26 @@
       </c>
       <c r="C1005" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1005" t="n">
-        <v>94.366</v>
+        <v>138.6</v>
       </c>
       <c r="E1005" t="n">
-        <v>94.733</v>
+        <v>138.8</v>
       </c>
       <c r="F1005" t="n">
-        <v>0.367</v>
+        <v>0.2</v>
       </c>
       <c r="G1005" t="n">
-        <v>5.531000000000001</v>
+        <v>3.767000000000001</v>
       </c>
     </row>
     <row r="1006">
       <c r="A1006" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1006" t="inlineStr">
@@ -29586,22 +29586,22 @@
         </is>
       </c>
       <c r="D1006" t="n">
-        <v>96.866</v>
+        <v>140.5</v>
       </c>
       <c r="E1006" t="n">
-        <v>97.366</v>
+        <v>140.7</v>
       </c>
       <c r="F1006" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G1006" t="n">
-        <v>6.031000000000001</v>
+        <v>3.967000000000001</v>
       </c>
     </row>
     <row r="1007">
       <c r="A1007" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1007" t="inlineStr">
@@ -29615,22 +29615,22 @@
         </is>
       </c>
       <c r="D1007" t="n">
-        <v>103.233</v>
+        <v>149.767</v>
       </c>
       <c r="E1007" t="n">
-        <v>103.8</v>
+        <v>149.967</v>
       </c>
       <c r="F1007" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="G1007" t="n">
-        <v>6.598000000000001</v>
+        <v>4.167000000000001</v>
       </c>
     </row>
     <row r="1008">
       <c r="A1008" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1008" t="inlineStr">
@@ -29640,26 +29640,26 @@
       </c>
       <c r="C1008" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1008" t="n">
-        <v>113.766</v>
+        <v>161.833</v>
       </c>
       <c r="E1008" t="n">
-        <v>114.533</v>
+        <v>162.033</v>
       </c>
       <c r="F1008" t="n">
-        <v>0.767</v>
+        <v>0.2</v>
       </c>
       <c r="G1008" t="n">
-        <v>7.365000000000001</v>
+        <v>4.367000000000001</v>
       </c>
     </row>
     <row r="1009">
       <c r="A1009" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1009" t="inlineStr">
@@ -29673,22 +29673,22 @@
         </is>
       </c>
       <c r="D1009" t="n">
-        <v>119.266</v>
+        <v>171.2</v>
       </c>
       <c r="E1009" t="n">
-        <v>120.733</v>
+        <v>171.533</v>
       </c>
       <c r="F1009" t="n">
-        <v>1.467</v>
+        <v>0.333</v>
       </c>
       <c r="G1009" t="n">
-        <v>8.832000000000001</v>
+        <v>4.700000000000001</v>
       </c>
     </row>
     <row r="1010">
       <c r="A1010" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1010" t="inlineStr">
@@ -29698,26 +29698,26 @@
       </c>
       <c r="C1010" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1010" t="n">
-        <v>123.433</v>
+        <v>172.233</v>
       </c>
       <c r="E1010" t="n">
-        <v>123.733</v>
+        <v>172.8</v>
       </c>
       <c r="F1010" t="n">
-        <v>0.3</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="G1010" t="n">
-        <v>9.132000000000001</v>
+        <v>5.267000000000001</v>
       </c>
     </row>
     <row r="1011">
       <c r="A1011" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1011" t="inlineStr">
@@ -29727,26 +29727,26 @@
       </c>
       <c r="C1011" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1011" t="n">
-        <v>126.233</v>
+        <v>181.333</v>
       </c>
       <c r="E1011" t="n">
-        <v>126.466</v>
+        <v>181.6</v>
       </c>
       <c r="F1011" t="n">
-        <v>0.233</v>
+        <v>0.267</v>
       </c>
       <c r="G1011" t="n">
-        <v>9.365000000000002</v>
+        <v>5.534000000000002</v>
       </c>
     </row>
     <row r="1012">
       <c r="A1012" t="inlineStr">
         <is>
-          <t>C50m3_test</t>
+          <t>c50m1_test</t>
         </is>
       </c>
       <c r="B1012" t="inlineStr">
@@ -29756,20 +29756,20 @@
       </c>
       <c r="C1012" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1012" t="n">
-        <v>129.333</v>
+        <v>197.967</v>
       </c>
       <c r="E1012" t="n">
-        <v>132.7</v>
+        <v>198.2</v>
       </c>
       <c r="F1012" t="n">
-        <v>3.367</v>
+        <v>0.233</v>
       </c>
       <c r="G1012" t="n">
-        <v>12.732</v>
+        <v>5.767000000000001</v>
       </c>
     </row>
     <row r="1013">
@@ -29789,16 +29789,16 @@
         </is>
       </c>
       <c r="D1013" t="n">
-        <v>5.267</v>
+        <v>214.6</v>
       </c>
       <c r="E1013" t="n">
-        <v>5.534</v>
+        <v>214.9</v>
       </c>
       <c r="F1013" t="n">
-        <v>0.267</v>
+        <v>0.3</v>
       </c>
       <c r="G1013" t="n">
-        <v>0.267</v>
+        <v>6.067000000000001</v>
       </c>
     </row>
     <row r="1014">
@@ -29814,20 +29814,20 @@
       </c>
       <c r="C1014" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1014" t="n">
-        <v>9.534000000000001</v>
+        <v>217.6</v>
       </c>
       <c r="E1014" t="n">
-        <v>10.067</v>
+        <v>217.867</v>
       </c>
       <c r="F1014" t="n">
-        <v>0.533</v>
+        <v>0.267</v>
       </c>
       <c r="G1014" t="n">
-        <v>0.8</v>
+        <v>6.334000000000001</v>
       </c>
     </row>
     <row r="1015">
@@ -29843,20 +29843,20 @@
       </c>
       <c r="C1015" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1015" t="n">
-        <v>21.634</v>
+        <v>218.8</v>
       </c>
       <c r="E1015" t="n">
-        <v>22.034</v>
+        <v>219</v>
       </c>
       <c r="F1015" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G1015" t="n">
-        <v>1.2</v>
+        <v>6.534000000000002</v>
       </c>
     </row>
     <row r="1016">
@@ -29876,16 +29876,16 @@
         </is>
       </c>
       <c r="D1016" t="n">
-        <v>42.1</v>
+        <v>231.733</v>
       </c>
       <c r="E1016" t="n">
-        <v>42.534</v>
+        <v>231.9</v>
       </c>
       <c r="F1016" t="n">
-        <v>0.434</v>
+        <v>0.167</v>
       </c>
       <c r="G1016" t="n">
-        <v>1.634</v>
+        <v>6.701000000000001</v>
       </c>
     </row>
     <row r="1017">
@@ -29905,16 +29905,16 @@
         </is>
       </c>
       <c r="D1017" t="n">
-        <v>56.234</v>
+        <v>233.767</v>
       </c>
       <c r="E1017" t="n">
-        <v>56.434</v>
+        <v>233.967</v>
       </c>
       <c r="F1017" t="n">
         <v>0.2</v>
       </c>
       <c r="G1017" t="n">
-        <v>1.834</v>
+        <v>6.901000000000002</v>
       </c>
     </row>
     <row r="1018">
@@ -29934,16 +29934,16 @@
         </is>
       </c>
       <c r="D1018" t="n">
-        <v>61.5</v>
+        <v>238.833</v>
       </c>
       <c r="E1018" t="n">
-        <v>62.534</v>
+        <v>239.233</v>
       </c>
       <c r="F1018" t="n">
-        <v>1.034</v>
+        <v>0.4</v>
       </c>
       <c r="G1018" t="n">
-        <v>2.868</v>
+        <v>7.301000000000002</v>
       </c>
     </row>
     <row r="1019">
@@ -29959,20 +29959,20 @@
       </c>
       <c r="C1019" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1019" t="n">
-        <v>90.73399999999999</v>
+        <v>241.933</v>
       </c>
       <c r="E1019" t="n">
-        <v>90.934</v>
+        <v>242.2</v>
       </c>
       <c r="F1019" t="n">
-        <v>0.2</v>
+        <v>0.267</v>
       </c>
       <c r="G1019" t="n">
-        <v>3.068000000000001</v>
+        <v>7.568000000000002</v>
       </c>
     </row>
     <row r="1020">
@@ -29992,16 +29992,16 @@
         </is>
       </c>
       <c r="D1020" t="n">
-        <v>122.767</v>
+        <v>244.933</v>
       </c>
       <c r="E1020" t="n">
-        <v>123.1</v>
+        <v>245.133</v>
       </c>
       <c r="F1020" t="n">
-        <v>0.333</v>
+        <v>0.2</v>
       </c>
       <c r="G1020" t="n">
-        <v>3.401000000000001</v>
+        <v>7.768000000000002</v>
       </c>
     </row>
     <row r="1021">
@@ -30017,20 +30017,20 @@
       </c>
       <c r="C1021" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1021" t="n">
-        <v>125.934</v>
+        <v>255.9</v>
       </c>
       <c r="E1021" t="n">
-        <v>126.1</v>
+        <v>256.1</v>
       </c>
       <c r="F1021" t="n">
-        <v>0.166</v>
+        <v>0.2</v>
       </c>
       <c r="G1021" t="n">
-        <v>3.567000000000001</v>
+        <v>7.968000000000003</v>
       </c>
     </row>
     <row r="1022">
@@ -30046,20 +30046,20 @@
       </c>
       <c r="C1022" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1022" t="n">
-        <v>138.6</v>
+        <v>260.4</v>
       </c>
       <c r="E1022" t="n">
-        <v>138.8</v>
+        <v>260.633</v>
       </c>
       <c r="F1022" t="n">
-        <v>0.2</v>
+        <v>0.233</v>
       </c>
       <c r="G1022" t="n">
-        <v>3.767000000000001</v>
+        <v>8.201000000000002</v>
       </c>
     </row>
     <row r="1023">
@@ -30079,16 +30079,16 @@
         </is>
       </c>
       <c r="D1023" t="n">
-        <v>140.5</v>
+        <v>301</v>
       </c>
       <c r="E1023" t="n">
-        <v>140.7</v>
+        <v>301.167</v>
       </c>
       <c r="F1023" t="n">
-        <v>0.2</v>
+        <v>0.167</v>
       </c>
       <c r="G1023" t="n">
-        <v>3.967000000000001</v>
+        <v>8.368000000000002</v>
       </c>
     </row>
     <row r="1024">
@@ -30104,20 +30104,20 @@
       </c>
       <c r="C1024" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1024" t="n">
-        <v>149.767</v>
+        <v>308.233</v>
       </c>
       <c r="E1024" t="n">
-        <v>149.967</v>
+        <v>308.4</v>
       </c>
       <c r="F1024" t="n">
-        <v>0.2</v>
+        <v>0.167</v>
       </c>
       <c r="G1024" t="n">
-        <v>4.167000000000001</v>
+        <v>8.535000000000002</v>
       </c>
     </row>
     <row r="1025">
@@ -30137,16 +30137,16 @@
         </is>
       </c>
       <c r="D1025" t="n">
-        <v>161.833</v>
+        <v>321.233</v>
       </c>
       <c r="E1025" t="n">
-        <v>162.033</v>
+        <v>321.733</v>
       </c>
       <c r="F1025" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="G1025" t="n">
-        <v>4.367000000000001</v>
+        <v>9.035000000000002</v>
       </c>
     </row>
     <row r="1026">
@@ -30162,20 +30162,20 @@
       </c>
       <c r="C1026" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1026" t="n">
-        <v>171.2</v>
+        <v>333.8</v>
       </c>
       <c r="E1026" t="n">
-        <v>171.533</v>
+        <v>334.3</v>
       </c>
       <c r="F1026" t="n">
-        <v>0.333</v>
+        <v>0.5</v>
       </c>
       <c r="G1026" t="n">
-        <v>4.700000000000001</v>
+        <v>9.535000000000002</v>
       </c>
     </row>
     <row r="1027">
@@ -30191,20 +30191,20 @@
       </c>
       <c r="C1027" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1027" t="n">
-        <v>172.233</v>
+        <v>334.967</v>
       </c>
       <c r="E1027" t="n">
-        <v>172.8</v>
+        <v>335.2</v>
       </c>
       <c r="F1027" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.233</v>
       </c>
       <c r="G1027" t="n">
-        <v>5.267000000000001</v>
+        <v>9.768000000000002</v>
       </c>
     </row>
     <row r="1028">
@@ -30220,20 +30220,20 @@
       </c>
       <c r="C1028" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1028" t="n">
-        <v>181.333</v>
+        <v>359.033</v>
       </c>
       <c r="E1028" t="n">
-        <v>181.6</v>
+        <v>359.233</v>
       </c>
       <c r="F1028" t="n">
-        <v>0.267</v>
+        <v>0.2</v>
       </c>
       <c r="G1028" t="n">
-        <v>5.534000000000002</v>
+        <v>9.968000000000002</v>
       </c>
     </row>
     <row r="1029">
@@ -30253,22 +30253,22 @@
         </is>
       </c>
       <c r="D1029" t="n">
-        <v>197.967</v>
+        <v>363.333</v>
       </c>
       <c r="E1029" t="n">
-        <v>198.2</v>
+        <v>363.533</v>
       </c>
       <c r="F1029" t="n">
-        <v>0.233</v>
+        <v>0.2</v>
       </c>
       <c r="G1029" t="n">
-        <v>5.767000000000001</v>
+        <v>10.168</v>
       </c>
     </row>
     <row r="1030">
       <c r="A1030" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1030" t="inlineStr">
@@ -30278,26 +30278,26 @@
       </c>
       <c r="C1030" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1030" t="n">
-        <v>214.6</v>
+        <v>10.766</v>
       </c>
       <c r="E1030" t="n">
-        <v>214.9</v>
+        <v>11.533</v>
       </c>
       <c r="F1030" t="n">
-        <v>0.3</v>
+        <v>0.767</v>
       </c>
       <c r="G1030" t="n">
-        <v>6.067000000000001</v>
+        <v>0.767</v>
       </c>
     </row>
     <row r="1031">
       <c r="A1031" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1031" t="inlineStr">
@@ -30311,22 +30311,22 @@
         </is>
       </c>
       <c r="D1031" t="n">
-        <v>217.6</v>
+        <v>18.133</v>
       </c>
       <c r="E1031" t="n">
-        <v>217.867</v>
+        <v>18.4</v>
       </c>
       <c r="F1031" t="n">
         <v>0.267</v>
       </c>
       <c r="G1031" t="n">
-        <v>6.334000000000001</v>
+        <v>1.034</v>
       </c>
     </row>
     <row r="1032">
       <c r="A1032" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1032" t="inlineStr">
@@ -30336,26 +30336,26 @@
       </c>
       <c r="C1032" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1032" t="n">
-        <v>218.8</v>
+        <v>26.866</v>
       </c>
       <c r="E1032" t="n">
-        <v>219</v>
+        <v>28.633</v>
       </c>
       <c r="F1032" t="n">
-        <v>0.2</v>
+        <v>1.767</v>
       </c>
       <c r="G1032" t="n">
-        <v>6.534000000000002</v>
+        <v>2.801</v>
       </c>
     </row>
     <row r="1033">
       <c r="A1033" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1033" t="inlineStr">
@@ -30369,22 +30369,22 @@
         </is>
       </c>
       <c r="D1033" t="n">
-        <v>231.733</v>
+        <v>33.6</v>
       </c>
       <c r="E1033" t="n">
-        <v>231.9</v>
+        <v>34.366</v>
       </c>
       <c r="F1033" t="n">
-        <v>0.167</v>
+        <v>0.766</v>
       </c>
       <c r="G1033" t="n">
-        <v>6.701000000000001</v>
+        <v>3.567</v>
       </c>
     </row>
     <row r="1034">
       <c r="A1034" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1034" t="inlineStr">
@@ -30394,26 +30394,26 @@
       </c>
       <c r="C1034" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1034" t="n">
-        <v>233.767</v>
+        <v>39.4</v>
       </c>
       <c r="E1034" t="n">
-        <v>233.967</v>
+        <v>41.4</v>
       </c>
       <c r="F1034" t="n">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="G1034" t="n">
-        <v>6.901000000000002</v>
+        <v>5.567</v>
       </c>
     </row>
     <row r="1035">
       <c r="A1035" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1035" t="inlineStr">
@@ -30427,22 +30427,22 @@
         </is>
       </c>
       <c r="D1035" t="n">
-        <v>238.833</v>
+        <v>47.3</v>
       </c>
       <c r="E1035" t="n">
-        <v>239.233</v>
+        <v>48.6</v>
       </c>
       <c r="F1035" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="G1035" t="n">
-        <v>7.301000000000002</v>
+        <v>6.867</v>
       </c>
     </row>
     <row r="1036">
       <c r="A1036" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1036" t="inlineStr">
@@ -30452,26 +30452,26 @@
       </c>
       <c r="C1036" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1036" t="n">
-        <v>241.933</v>
+        <v>58.766</v>
       </c>
       <c r="E1036" t="n">
-        <v>242.2</v>
+        <v>59.466</v>
       </c>
       <c r="F1036" t="n">
-        <v>0.267</v>
+        <v>0.7</v>
       </c>
       <c r="G1036" t="n">
-        <v>7.568000000000002</v>
+        <v>7.567</v>
       </c>
     </row>
     <row r="1037">
       <c r="A1037" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1037" t="inlineStr">
@@ -30481,26 +30481,26 @@
       </c>
       <c r="C1037" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1037" t="n">
-        <v>244.933</v>
+        <v>61.433</v>
       </c>
       <c r="E1037" t="n">
-        <v>245.133</v>
+        <v>63.266</v>
       </c>
       <c r="F1037" t="n">
-        <v>0.2</v>
+        <v>1.833</v>
       </c>
       <c r="G1037" t="n">
-        <v>7.768000000000002</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="1038">
       <c r="A1038" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1038" t="inlineStr">
@@ -30514,22 +30514,22 @@
         </is>
       </c>
       <c r="D1038" t="n">
-        <v>255.9</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="E1038" t="n">
-        <v>256.1</v>
+        <v>65.46599999999999</v>
       </c>
       <c r="F1038" t="n">
-        <v>0.2</v>
+        <v>0.366</v>
       </c>
       <c r="G1038" t="n">
-        <v>7.968000000000003</v>
+        <v>9.766</v>
       </c>
     </row>
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m2_test</t>
         </is>
       </c>
       <c r="B1039" t="inlineStr">
@@ -30539,26 +30539,26 @@
       </c>
       <c r="C1039" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1039" t="n">
-        <v>260.4</v>
+        <v>70.533</v>
       </c>
       <c r="E1039" t="n">
-        <v>260.633</v>
+        <v>70.8</v>
       </c>
       <c r="F1039" t="n">
-        <v>0.233</v>
+        <v>0.267</v>
       </c>
       <c r="G1039" t="n">
-        <v>8.201000000000002</v>
+        <v>10.033</v>
       </c>
     </row>
     <row r="1040">
       <c r="A1040" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1040" t="inlineStr">
@@ -30568,26 +30568,26 @@
       </c>
       <c r="C1040" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1040" t="n">
-        <v>301</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E1040" t="n">
-        <v>301.167</v>
+        <v>9.566000000000001</v>
       </c>
       <c r="F1040" t="n">
-        <v>0.167</v>
+        <v>0.266</v>
       </c>
       <c r="G1040" t="n">
-        <v>8.368000000000002</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="1041">
       <c r="A1041" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1041" t="inlineStr">
@@ -30597,26 +30597,26 @@
       </c>
       <c r="C1041" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1041" t="n">
-        <v>308.233</v>
+        <v>12.7</v>
       </c>
       <c r="E1041" t="n">
-        <v>308.4</v>
+        <v>12.866</v>
       </c>
       <c r="F1041" t="n">
-        <v>0.167</v>
+        <v>0.166</v>
       </c>
       <c r="G1041" t="n">
-        <v>8.535000000000002</v>
+        <v>0.4320000000000001</v>
       </c>
     </row>
     <row r="1042">
       <c r="A1042" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1042" t="inlineStr">
@@ -30630,22 +30630,22 @@
         </is>
       </c>
       <c r="D1042" t="n">
-        <v>321.233</v>
+        <v>28.033</v>
       </c>
       <c r="E1042" t="n">
-        <v>321.733</v>
+        <v>28.366</v>
       </c>
       <c r="F1042" t="n">
-        <v>0.5</v>
+        <v>0.333</v>
       </c>
       <c r="G1042" t="n">
-        <v>9.035000000000002</v>
+        <v>0.7650000000000001</v>
       </c>
     </row>
     <row r="1043">
       <c r="A1043" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1043" t="inlineStr">
@@ -30655,26 +30655,26 @@
       </c>
       <c r="C1043" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1043" t="n">
-        <v>333.8</v>
+        <v>32.266</v>
       </c>
       <c r="E1043" t="n">
-        <v>334.3</v>
+        <v>33.366</v>
       </c>
       <c r="F1043" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="G1043" t="n">
-        <v>9.535000000000002</v>
+        <v>1.865</v>
       </c>
     </row>
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1044" t="inlineStr">
@@ -30684,26 +30684,26 @@
       </c>
       <c r="C1044" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1044" t="n">
-        <v>334.967</v>
+        <v>37.733</v>
       </c>
       <c r="E1044" t="n">
-        <v>335.2</v>
+        <v>37.966</v>
       </c>
       <c r="F1044" t="n">
         <v>0.233</v>
       </c>
       <c r="G1044" t="n">
-        <v>9.768000000000002</v>
+        <v>2.098</v>
       </c>
     </row>
     <row r="1045">
       <c r="A1045" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1045" t="inlineStr">
@@ -30713,26 +30713,26 @@
       </c>
       <c r="C1045" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1045" t="n">
-        <v>359.033</v>
+        <v>50.166</v>
       </c>
       <c r="E1045" t="n">
-        <v>359.233</v>
+        <v>50.966</v>
       </c>
       <c r="F1045" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="G1045" t="n">
-        <v>9.968000000000002</v>
+        <v>2.898000000000001</v>
       </c>
     </row>
     <row r="1046">
       <c r="A1046" t="inlineStr">
         <is>
-          <t>c50m1_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1046" t="inlineStr">
@@ -30742,26 +30742,26 @@
       </c>
       <c r="C1046" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1046" t="n">
-        <v>363.333</v>
+        <v>57.333</v>
       </c>
       <c r="E1046" t="n">
-        <v>363.533</v>
+        <v>58.266</v>
       </c>
       <c r="F1046" t="n">
-        <v>0.2</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="G1046" t="n">
-        <v>10.168</v>
+        <v>3.831</v>
       </c>
     </row>
     <row r="1047">
       <c r="A1047" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1047" t="inlineStr">
@@ -30771,26 +30771,26 @@
       </c>
       <c r="C1047" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1047" t="n">
-        <v>10.766</v>
+        <v>62.433</v>
       </c>
       <c r="E1047" t="n">
-        <v>11.533</v>
+        <v>63.366</v>
       </c>
       <c r="F1047" t="n">
-        <v>0.767</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="G1047" t="n">
-        <v>0.767</v>
+        <v>4.764</v>
       </c>
     </row>
     <row r="1048">
       <c r="A1048" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1048" t="inlineStr">
@@ -30804,22 +30804,22 @@
         </is>
       </c>
       <c r="D1048" t="n">
-        <v>18.133</v>
+        <v>82</v>
       </c>
       <c r="E1048" t="n">
-        <v>18.4</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="F1048" t="n">
-        <v>0.267</v>
+        <v>0.4</v>
       </c>
       <c r="G1048" t="n">
-        <v>1.034</v>
+        <v>5.164000000000001</v>
       </c>
     </row>
     <row r="1049">
       <c r="A1049" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1049" t="inlineStr">
@@ -30833,22 +30833,22 @@
         </is>
       </c>
       <c r="D1049" t="n">
-        <v>26.866</v>
+        <v>94.366</v>
       </c>
       <c r="E1049" t="n">
-        <v>28.633</v>
+        <v>94.733</v>
       </c>
       <c r="F1049" t="n">
-        <v>1.767</v>
+        <v>0.367</v>
       </c>
       <c r="G1049" t="n">
-        <v>2.801</v>
+        <v>5.531000000000001</v>
       </c>
     </row>
     <row r="1050">
       <c r="A1050" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1050" t="inlineStr">
@@ -30858,26 +30858,26 @@
       </c>
       <c r="C1050" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1050" t="n">
-        <v>33.6</v>
+        <v>96.866</v>
       </c>
       <c r="E1050" t="n">
-        <v>34.366</v>
+        <v>97.366</v>
       </c>
       <c r="F1050" t="n">
-        <v>0.766</v>
+        <v>0.5</v>
       </c>
       <c r="G1050" t="n">
-        <v>3.567</v>
+        <v>6.031000000000001</v>
       </c>
     </row>
     <row r="1051">
       <c r="A1051" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1051" t="inlineStr">
@@ -30887,26 +30887,26 @@
       </c>
       <c r="C1051" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1051" t="n">
-        <v>39.4</v>
+        <v>103.233</v>
       </c>
       <c r="E1051" t="n">
-        <v>41.4</v>
+        <v>103.8</v>
       </c>
       <c r="F1051" t="n">
-        <v>2</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="G1051" t="n">
-        <v>5.567</v>
+        <v>6.598000000000001</v>
       </c>
     </row>
     <row r="1052">
       <c r="A1052" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1052" t="inlineStr">
@@ -30920,22 +30920,22 @@
         </is>
       </c>
       <c r="D1052" t="n">
-        <v>47.3</v>
+        <v>113.766</v>
       </c>
       <c r="E1052" t="n">
-        <v>48.6</v>
+        <v>114.533</v>
       </c>
       <c r="F1052" t="n">
-        <v>1.3</v>
+        <v>0.767</v>
       </c>
       <c r="G1052" t="n">
-        <v>6.867</v>
+        <v>7.365000000000001</v>
       </c>
     </row>
     <row r="1053">
       <c r="A1053" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1053" t="inlineStr">
@@ -30945,26 +30945,26 @@
       </c>
       <c r="C1053" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1053" t="n">
-        <v>58.766</v>
+        <v>119.266</v>
       </c>
       <c r="E1053" t="n">
-        <v>59.466</v>
+        <v>120.733</v>
       </c>
       <c r="F1053" t="n">
-        <v>0.7</v>
+        <v>1.467</v>
       </c>
       <c r="G1053" t="n">
-        <v>7.567</v>
+        <v>8.832000000000001</v>
       </c>
     </row>
     <row r="1054">
       <c r="A1054" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1054" t="inlineStr">
@@ -30974,26 +30974,26 @@
       </c>
       <c r="C1054" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1054" t="n">
-        <v>61.433</v>
+        <v>123.433</v>
       </c>
       <c r="E1054" t="n">
-        <v>63.266</v>
+        <v>123.733</v>
       </c>
       <c r="F1054" t="n">
-        <v>1.833</v>
+        <v>0.3</v>
       </c>
       <c r="G1054" t="n">
-        <v>9.4</v>
+        <v>9.132000000000001</v>
       </c>
     </row>
     <row r="1055">
       <c r="A1055" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1055" t="inlineStr">
@@ -31003,26 +31003,26 @@
       </c>
       <c r="C1055" t="inlineStr">
         <is>
-          <t>Explore_N</t>
+          <t>Explore_F</t>
         </is>
       </c>
       <c r="D1055" t="n">
-        <v>65.09999999999999</v>
+        <v>126.233</v>
       </c>
       <c r="E1055" t="n">
-        <v>65.46599999999999</v>
+        <v>126.466</v>
       </c>
       <c r="F1055" t="n">
-        <v>0.366</v>
+        <v>0.233</v>
       </c>
       <c r="G1055" t="n">
-        <v>9.766</v>
+        <v>9.365000000000002</v>
       </c>
     </row>
     <row r="1056">
       <c r="A1056" t="inlineStr">
         <is>
-          <t>c50m2_test</t>
+          <t>c50m3_test</t>
         </is>
       </c>
       <c r="B1056" t="inlineStr">
@@ -31032,20 +31032,20 @@
       </c>
       <c r="C1056" t="inlineStr">
         <is>
-          <t>Explore_F</t>
+          <t>Explore_N</t>
         </is>
       </c>
       <c r="D1056" t="n">
-        <v>70.533</v>
+        <v>129.333</v>
       </c>
       <c r="E1056" t="n">
-        <v>70.8</v>
+        <v>132.7</v>
       </c>
       <c r="F1056" t="n">
-        <v>0.267</v>
+        <v>3.367</v>
       </c>
       <c r="G1056" t="n">
-        <v>10.033</v>
+        <v>12.732</v>
       </c>
     </row>
     <row r="1057">

</xml_diff>